<commit_message>
fix: add ARR tab to demand_plan_template.xlsx, remove standalone ARR_template
- ARR sheet added directly to existing demand_plan_template.xlsx
  (Month | Monthly Target (€) | Monthly Actual (€), Jan–Dec)
- Removed separate ARR_template.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demand_plan_template.xlsx
+++ b/demand_plan_template.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="€#,##0;(€#,##0);-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,8 +82,30 @@
       <color rgb="0010FBCF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0064B5F6"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00A0AEC0"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -124,8 +147,28 @@
         <fgColor rgb="00FFFDE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1A2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D2D44"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0016213E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F3460"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -194,11 +237,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="003A3A5C"/>
+      </left>
+      <right style="thin">
+        <color rgb="003A3A5C"/>
+      </right>
+      <top style="thin">
+        <color rgb="003A3A5C"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="003A3A5C"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -303,6 +360,24 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1393,4 +1468,190 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>ARR Forecast — 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="38" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B2" s="38" t="inlineStr">
+        <is>
+          <t>Monthly Target (€)</t>
+        </is>
+      </c>
+      <c r="C2" s="38" t="inlineStr">
+        <is>
+          <t>Monthly Actual (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C3" s="41" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C4" s="41" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="39" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C5" s="41" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="39" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C6" s="41" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C7" s="41" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="39" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C8" s="41" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="39" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C9" s="41" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="39" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C10" s="41" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C11" s="41" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C12" s="41" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C13" s="41" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C14" s="41" t="n"/>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="42" t="inlineStr">
+        <is>
+          <t>Instructions: Fill in Monthly Actual (€) as each month closes. Column B = monthly ARR new bookings target. The dashboard auto-computes a reforecast trajectory from your actuals.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>